<commit_message>
Added JCalendar and improved Lecture Attendance
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -334,7 +334,7 @@
         <v>45959.0</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>16</v>
@@ -351,7 +351,7 @@
         <v>45959.0</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>16</v>

</xml_diff>

<commit_message>
Added Sort for columns
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="25">
   <si>
     <t>ID</t>
   </si>
@@ -50,6 +50,30 @@
   </si>
   <si>
     <t>Мосейко Роман Адреевич</t>
+  </si>
+  <si>
+    <t>Маленков Станислав Владимирович</t>
+  </si>
+  <si>
+    <t>Живоглод Никита Андреевич</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Антоненко Дмитрий </t>
+  </si>
+  <si>
+    <t>Бородейко Яна Максимовна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вечерко Полина </t>
+  </si>
+  <si>
+    <t>Грушко Анастасия Юрьевна</t>
+  </si>
+  <si>
+    <t>Журов Ярослав</t>
+  </si>
+  <si>
+    <t>Глинский Никита Александрович</t>
   </si>
   <si>
     <t>Дата</t>
@@ -184,7 +208,7 @@
         <v>4</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>3.0</v>
+        <v>11.0</v>
       </c>
     </row>
   </sheetData>
@@ -194,11 +218,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.6171875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="29.0546875" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="31.62109375" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.21875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="17.20703125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="11.87890625" customWidth="true" bestFit="true"/>
@@ -235,7 +259,7 @@
         <v>4</v>
       </c>
       <c r="E2" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="3">
@@ -252,7 +276,7 @@
         <v>4</v>
       </c>
       <c r="E3" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="4">
@@ -269,6 +293,142 @@
         <v>4</v>
       </c>
       <c r="E4" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="0">
+        <v>3.0</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C5" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E5" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n" s="0">
+        <v>4.0</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="C6" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E6" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="C7" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E7" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n" s="0">
+        <v>6.0</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="C8" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E8" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="C9" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E9" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n" s="0">
+        <v>8.0</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C10" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E10" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n" s="0">
+        <v>9.0</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="C11" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E11" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n" s="0">
+        <v>10.0</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C12" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E12" t="n" s="0">
         <v>1.0</v>
       </c>
     </row>
@@ -279,13 +439,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="10.21875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="17.20703125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="9.92578125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="29.0546875" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="31.62109375" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="14.71875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -297,13 +457,13 @@
         <v>1</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s" s="1">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>14</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2">
@@ -320,7 +480,7 @@
         <v>9</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>15</v>
+        <v>23</v>
       </c>
     </row>
     <row r="3">
@@ -334,10 +494,10 @@
         <v>45959.0</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>16</v>
+        <v>23</v>
       </c>
     </row>
     <row r="4">
@@ -351,10 +511,197 @@
         <v>45959.0</v>
       </c>
       <c r="D4" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C13" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D13" t="s" s="0">
         <v>10</v>
       </c>
-      <c r="E4" t="s" s="0">
-        <v>16</v>
+      <c r="E13" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C14" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n" s="2">
+        <v>45960.0</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixing ReportPanel - only chosen group
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -477,7 +477,7 @@
         <v>45959.0</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>23</v>
@@ -494,7 +494,7 @@
         <v>45959.0</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>23</v>
@@ -528,7 +528,7 @@
         <v>45960.0</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>18</v>
+        <v>11</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>23</v>
@@ -545,10 +545,10 @@
         <v>45960.0</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="7">
@@ -562,7 +562,7 @@
         <v>45960.0</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>23</v>
@@ -579,10 +579,10 @@
         <v>45960.0</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -596,10 +596,10 @@
         <v>45960.0</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="10">
@@ -613,10 +613,10 @@
         <v>45960.0</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="11">
@@ -630,10 +630,10 @@
         <v>45960.0</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="12">
@@ -647,7 +647,7 @@
         <v>45960.0</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E12" t="s" s="0">
         <v>23</v>
@@ -664,7 +664,7 @@
         <v>45960.0</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E13" t="s" s="0">
         <v>23</v>
@@ -681,10 +681,10 @@
         <v>45960.0</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="15">
@@ -698,7 +698,7 @@
         <v>45960.0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E15" t="s" s="0">
         <v>23</v>

</xml_diff>

<commit_message>
Added Export to Excel from ReportPanel && fixed bug with edit and deleting rows in StudepntPanel
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="29">
   <si>
     <t>ID</t>
   </si>
@@ -41,6 +41,18 @@
   </si>
   <si>
     <t>Посещений</t>
+  </si>
+  <si>
+    <t>Вика (Староста)</t>
+  </si>
+  <si>
+    <t>Пустошило Алексей</t>
+  </si>
+  <si>
+    <t>Кадебская Карина</t>
+  </si>
+  <si>
+    <t>Пивоварчик Максим</t>
   </si>
   <si>
     <t>Борсук Ростислав Александрович</t>
@@ -197,7 +209,7 @@
         <v>3</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="3">
@@ -218,7 +230,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.6171875" customWidth="true" bestFit="true"/>
@@ -253,13 +265,13 @@
         <v>9</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E2" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="3">
@@ -270,10 +282,10 @@
         <v>10</v>
       </c>
       <c r="C3" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n" s="0">
         <v>0.0</v>
@@ -287,10 +299,10 @@
         <v>11</v>
       </c>
       <c r="C4" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E4" t="n" s="0">
         <v>0.0</v>
@@ -304,10 +316,10 @@
         <v>12</v>
       </c>
       <c r="C5" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n" s="0">
         <v>0.0</v>
@@ -327,7 +339,7 @@
         <v>4</v>
       </c>
       <c r="E6" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="7">
@@ -344,7 +356,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="8">
@@ -412,7 +424,7 @@
         <v>4</v>
       </c>
       <c r="E11" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="12">
@@ -429,6 +441,74 @@
         <v>4</v>
       </c>
       <c r="E12" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n" s="0">
+        <v>11.0</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="C13" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E13" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n" s="0">
+        <v>12.0</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="C14" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E14" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n" s="0">
+        <v>13.0</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C15" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E15" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n" s="0">
+        <v>14.0</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="C16" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E16" t="n" s="0">
         <v>1.0</v>
       </c>
     </row>
@@ -457,13 +537,13 @@
         <v>1</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D1" t="s" s="1">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2">
@@ -477,10 +557,10 @@
         <v>45959.0</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3">
@@ -494,10 +574,10 @@
         <v>45959.0</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4">
@@ -511,10 +591,10 @@
         <v>45959.0</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
@@ -528,10 +608,10 @@
         <v>45960.0</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -545,10 +625,10 @@
         <v>45960.0</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="7">
@@ -562,10 +642,10 @@
         <v>45960.0</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="8">
@@ -579,10 +659,10 @@
         <v>45960.0</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -596,10 +676,10 @@
         <v>45960.0</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>23</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
@@ -616,7 +696,7 @@
         <v>15</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11">
@@ -630,10 +710,10 @@
         <v>45960.0</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="12">
@@ -647,10 +727,10 @@
         <v>45960.0</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13">
@@ -664,10 +744,10 @@
         <v>45960.0</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>23</v>
+        <v>27</v>
       </c>
     </row>
     <row r="14">
@@ -684,7 +764,7 @@
         <v>19</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
@@ -698,10 +778,10 @@
         <v>45960.0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed Bug with delete group in GroupPanel
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="29">
   <si>
     <t>ID</t>
   </si>
@@ -356,7 +356,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="8">
@@ -373,7 +373,7 @@
         <v>4</v>
       </c>
       <c r="E8" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="9">
@@ -407,7 +407,7 @@
         <v>4</v>
       </c>
       <c r="E10" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="11">
@@ -441,7 +441,7 @@
         <v>4</v>
       </c>
       <c r="E12" t="n" s="0">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="13">
@@ -519,7 +519,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E48"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="10.21875" customWidth="true" bestFit="true"/>
@@ -642,7 +642,7 @@
         <v>45960.0</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>27</v>
@@ -659,10 +659,10 @@
         <v>45960.0</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9">
@@ -676,10 +676,10 @@
         <v>45960.0</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10">
@@ -693,10 +693,10 @@
         <v>45960.0</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11">
@@ -710,10 +710,10 @@
         <v>45960.0</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12">
@@ -744,7 +744,7 @@
         <v>45960.0</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E13" t="s" s="0">
         <v>27</v>
@@ -761,7 +761,7 @@
         <v>45960.0</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E14" t="s" s="0">
         <v>27</v>
@@ -778,10 +778,571 @@
         <v>45960.0</v>
       </c>
       <c r="D15" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C16" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C17" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C18" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C19" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C20" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C21" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C22" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C23" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D23" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E23" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C24" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D24" t="s" s="0">
         <v>14</v>
       </c>
-      <c r="E15" t="s" s="0">
-        <v>27</v>
+      <c r="E24" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D25" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E25" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C26" t="n" s="2">
+        <v>45951.0</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E26" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D27" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E27" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C28" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C29" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D29" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E29" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C30" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D30" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E30" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C31" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D31" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E31" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C32" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C33" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D33" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E33" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C34" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D34" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E34" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C35" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D35" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E35" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C36" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D36" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E36" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C37" t="n" s="2">
+        <v>45957.0</v>
+      </c>
+      <c r="D37" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E37" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C38" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D38" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E38" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C39" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D39" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E39" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C40" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D40" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E40" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C41" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D41" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E41" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B42" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C42" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D42" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E42" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C43" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D43" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="E43" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C44" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D44" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E44" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C45" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D45" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E45" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C46" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D46" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E46" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C47" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D47" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E47" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C48" t="n" s="2">
+        <v>45961.0</v>
+      </c>
+      <c r="D48" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E48" t="s" s="0">
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added ToolTips on Buttons :)
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -557,7 +557,7 @@
         <v>45959.0</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>27</v>
@@ -574,7 +574,7 @@
         <v>45959.0</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>27</v>
@@ -591,7 +591,7 @@
         <v>45959.0</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>27</v>
@@ -608,7 +608,7 @@
         <v>45960.0</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>27</v>
@@ -625,10 +625,10 @@
         <v>45960.0</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
@@ -642,7 +642,7 @@
         <v>45960.0</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>27</v>
@@ -676,7 +676,7 @@
         <v>45960.0</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E9" t="s" s="0">
         <v>27</v>
@@ -693,10 +693,10 @@
         <v>45960.0</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         <v>45960.0</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E11" t="s" s="0">
         <v>27</v>
@@ -727,7 +727,7 @@
         <v>45960.0</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E12" t="s" s="0">
         <v>27</v>
@@ -744,10 +744,10 @@
         <v>45960.0</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14">
@@ -761,10 +761,10 @@
         <v>45960.0</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="15">
@@ -778,7 +778,7 @@
         <v>45960.0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E15" t="s" s="0">
         <v>27</v>
@@ -795,10 +795,10 @@
         <v>45951.0</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
@@ -812,7 +812,7 @@
         <v>45951.0</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="E17" t="s" s="0">
         <v>27</v>
@@ -829,7 +829,7 @@
         <v>45951.0</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E18" t="s" s="0">
         <v>28</v>
@@ -863,10 +863,10 @@
         <v>45951.0</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="21">
@@ -880,10 +880,10 @@
         <v>45951.0</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22">
@@ -897,7 +897,7 @@
         <v>45951.0</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E22" t="s" s="0">
         <v>27</v>
@@ -914,10 +914,10 @@
         <v>45951.0</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24">
@@ -931,10 +931,10 @@
         <v>45951.0</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="25">
@@ -948,7 +948,7 @@
         <v>45951.0</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E25" t="s" s="0">
         <v>27</v>
@@ -965,10 +965,10 @@
         <v>45951.0</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="27">
@@ -982,7 +982,7 @@
         <v>45957.0</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E27" t="s" s="0">
         <v>27</v>
@@ -999,7 +999,7 @@
         <v>45957.0</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="E28" t="s" s="0">
         <v>27</v>
@@ -1016,10 +1016,10 @@
         <v>45957.0</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E29" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="30">
@@ -1050,7 +1050,7 @@
         <v>45957.0</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E31" t="s" s="0">
         <v>27</v>
@@ -1067,10 +1067,10 @@
         <v>45957.0</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E32" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="33">
@@ -1084,7 +1084,7 @@
         <v>45957.0</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E33" t="s" s="0">
         <v>27</v>
@@ -1101,7 +1101,7 @@
         <v>45957.0</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E34" t="s" s="0">
         <v>27</v>
@@ -1118,7 +1118,7 @@
         <v>45957.0</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E35" t="s" s="0">
         <v>27</v>
@@ -1135,7 +1135,7 @@
         <v>45957.0</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E36" t="s" s="0">
         <v>27</v>
@@ -1152,7 +1152,7 @@
         <v>45957.0</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E37" t="s" s="0">
         <v>27</v>
@@ -1169,7 +1169,7 @@
         <v>45961.0</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E38" t="s" s="0">
         <v>27</v>
@@ -1186,7 +1186,7 @@
         <v>45961.0</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="E39" t="s" s="0">
         <v>27</v>
@@ -1203,10 +1203,10 @@
         <v>45961.0</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="41">
@@ -1237,7 +1237,7 @@
         <v>45961.0</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E42" t="s" s="0">
         <v>27</v>
@@ -1254,10 +1254,10 @@
         <v>45961.0</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="E43" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="44">
@@ -1271,7 +1271,7 @@
         <v>45961.0</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E44" t="s" s="0">
         <v>27</v>
@@ -1288,7 +1288,7 @@
         <v>45961.0</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="E45" t="s" s="0">
         <v>27</v>
@@ -1305,7 +1305,7 @@
         <v>45961.0</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="E46" t="s" s="0">
         <v>27</v>
@@ -1322,7 +1322,7 @@
         <v>45961.0</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c r="E47" t="s" s="0">
         <v>27</v>
@@ -1339,7 +1339,7 @@
         <v>45961.0</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="E48" t="s" s="0">
         <v>27</v>

</xml_diff>

<commit_message>
Added Timer in Bottim Grid
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -574,7 +574,7 @@
         <v>45959.0</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E3" t="s" s="0">
         <v>27</v>
@@ -591,7 +591,7 @@
         <v>45959.0</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>27</v>
@@ -608,7 +608,7 @@
         <v>45960.0</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>27</v>
@@ -642,7 +642,7 @@
         <v>45960.0</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>28</v>
@@ -659,7 +659,7 @@
         <v>45960.0</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E8" t="s" s="0">
         <v>27</v>
@@ -693,10 +693,10 @@
         <v>45960.0</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="11">
@@ -710,7 +710,7 @@
         <v>45960.0</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E11" t="s" s="0">
         <v>27</v>
@@ -727,10 +727,10 @@
         <v>45960.0</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="13">
@@ -744,10 +744,10 @@
         <v>45960.0</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14">
@@ -761,10 +761,10 @@
         <v>45960.0</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15">
@@ -778,7 +778,7 @@
         <v>45960.0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E15" t="s" s="0">
         <v>27</v>
@@ -795,7 +795,7 @@
         <v>45951.0</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E16" t="s" s="0">
         <v>27</v>
@@ -829,7 +829,7 @@
         <v>45951.0</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E18" t="s" s="0">
         <v>27</v>
@@ -846,10 +846,10 @@
         <v>45951.0</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="20">
@@ -880,10 +880,10 @@
         <v>45951.0</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22">
@@ -897,7 +897,7 @@
         <v>45951.0</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E22" t="s" s="0">
         <v>28</v>
@@ -914,7 +914,7 @@
         <v>45951.0</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E23" t="s" s="0">
         <v>27</v>
@@ -931,7 +931,7 @@
         <v>45951.0</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E24" t="s" s="0">
         <v>27</v>
@@ -948,10 +948,10 @@
         <v>45951.0</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="26">
@@ -965,10 +965,10 @@
         <v>45951.0</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27">
@@ -982,7 +982,7 @@
         <v>45957.0</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E27" t="s" s="0">
         <v>27</v>
@@ -1016,7 +1016,7 @@
         <v>45957.0</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E29" t="s" s="0">
         <v>27</v>
@@ -1033,7 +1033,7 @@
         <v>45957.0</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E30" t="s" s="0">
         <v>27</v>
@@ -1067,7 +1067,7 @@
         <v>45957.0</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="E32" t="s" s="0">
         <v>27</v>
@@ -1084,7 +1084,7 @@
         <v>45957.0</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E33" t="s" s="0">
         <v>27</v>
@@ -1101,7 +1101,7 @@
         <v>45957.0</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E34" t="s" s="0">
         <v>27</v>
@@ -1118,7 +1118,7 @@
         <v>45957.0</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E35" t="s" s="0">
         <v>27</v>
@@ -1135,7 +1135,7 @@
         <v>45957.0</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E36" t="s" s="0">
         <v>27</v>
@@ -1152,7 +1152,7 @@
         <v>45957.0</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E37" t="s" s="0">
         <v>27</v>
@@ -1169,7 +1169,7 @@
         <v>45961.0</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E38" t="s" s="0">
         <v>27</v>
@@ -1203,7 +1203,7 @@
         <v>45961.0</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="E40" t="s" s="0">
         <v>27</v>
@@ -1220,7 +1220,7 @@
         <v>45961.0</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E41" t="s" s="0">
         <v>27</v>
@@ -1254,7 +1254,7 @@
         <v>45961.0</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="E43" t="s" s="0">
         <v>27</v>
@@ -1271,7 +1271,7 @@
         <v>45961.0</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E44" t="s" s="0">
         <v>27</v>
@@ -1288,7 +1288,7 @@
         <v>45961.0</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="E45" t="s" s="0">
         <v>27</v>
@@ -1305,7 +1305,7 @@
         <v>45961.0</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="E46" t="s" s="0">
         <v>27</v>
@@ -1322,7 +1322,7 @@
         <v>45961.0</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E47" t="s" s="0">
         <v>27</v>
@@ -1339,7 +1339,7 @@
         <v>45961.0</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="E48" t="s" s="0">
         <v>27</v>

</xml_diff>

<commit_message>
Added Percents for Attendance
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="48">
   <si>
     <t>ID</t>
   </si>
@@ -152,6 +152,12 @@
   </si>
   <si>
     <t>Присутствовал</t>
+  </si>
+  <si>
+    <t>Да</t>
+  </si>
+  <si>
+    <t>Нет</t>
   </si>
 </sst>
 </file>
@@ -407,7 +413,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="8">
@@ -441,7 +447,7 @@
         <v>4</v>
       </c>
       <c r="E9" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="10">
@@ -458,7 +464,7 @@
         <v>4</v>
       </c>
       <c r="E10" t="n" s="0">
-        <v>0.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="11">
@@ -475,7 +481,7 @@
         <v>4</v>
       </c>
       <c r="E11" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="12">
@@ -492,7 +498,7 @@
         <v>4</v>
       </c>
       <c r="E12" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="13">
@@ -509,7 +515,7 @@
         <v>4</v>
       </c>
       <c r="E13" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="14">
@@ -526,7 +532,7 @@
         <v>4</v>
       </c>
       <c r="E14" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="15">
@@ -543,7 +549,7 @@
         <v>4</v>
       </c>
       <c r="E15" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="16">
@@ -560,7 +566,7 @@
         <v>4</v>
       </c>
       <c r="E16" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="17">
@@ -577,7 +583,7 @@
         <v>4</v>
       </c>
       <c r="E17" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="18">
@@ -594,7 +600,7 @@
         <v>4</v>
       </c>
       <c r="E18" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="19">
@@ -611,7 +617,7 @@
         <v>4</v>
       </c>
       <c r="E19" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="20">
@@ -628,7 +634,7 @@
         <v>4</v>
       </c>
       <c r="E20" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="21">
@@ -645,7 +651,7 @@
         <v>4</v>
       </c>
       <c r="E21" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="22">
@@ -662,7 +668,7 @@
         <v>4</v>
       </c>
       <c r="E22" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="23">
@@ -679,7 +685,7 @@
         <v>4</v>
       </c>
       <c r="E23" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="24">
@@ -696,7 +702,7 @@
         <v>4</v>
       </c>
       <c r="E24" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="25">
@@ -713,7 +719,7 @@
         <v>4</v>
       </c>
       <c r="E25" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="26">
@@ -730,7 +736,7 @@
         <v>4</v>
       </c>
       <c r="E26" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="27">
@@ -747,7 +753,7 @@
         <v>4</v>
       </c>
       <c r="E27" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="28">
@@ -764,7 +770,7 @@
         <v>4</v>
       </c>
       <c r="E28" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="29">
@@ -781,7 +787,7 @@
         <v>4</v>
       </c>
       <c r="E29" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="30">
@@ -798,7 +804,7 @@
         <v>4</v>
       </c>
       <c r="E30" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="31">
@@ -815,7 +821,7 @@
         <v>4</v>
       </c>
       <c r="E31" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="32">
@@ -832,7 +838,7 @@
         <v>4</v>
       </c>
       <c r="E32" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
     <row r="33">
@@ -849,7 +855,7 @@
         <v>4</v>
       </c>
       <c r="E33" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="34">
@@ -883,7 +889,7 @@
         <v>4</v>
       </c>
       <c r="E35" t="n" s="0">
-        <v>0.0</v>
+        <v>4.0</v>
       </c>
     </row>
   </sheetData>
@@ -893,13 +899,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="10.21875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="17.20703125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="14.10546875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="9.92578125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="32.01953125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="14.71875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -920,6 +926,2046 @@
         <v>45</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C13" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C14" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C16" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C17" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C18" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C19" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C20" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C21" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C22" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C23" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D23" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E23" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C24" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D24" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E24" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D25" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E25" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C26" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="E26" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D27" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E27" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C28" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C29" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D29" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E29" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C30" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D30" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E30" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C31" t="n" s="2">
+        <v>45903.0</v>
+      </c>
+      <c r="D31" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E31" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B32" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C32" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D32" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E32" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B33" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C33" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D33" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="E33" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B34" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C34" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D34" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E34" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B35" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C35" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D35" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="E35" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C36" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D36" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E36" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C37" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D37" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E37" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C38" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D38" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E38" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C39" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D39" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E39" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C40" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D40" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E40" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C41" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D41" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E41" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B42" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C42" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D42" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E42" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C43" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D43" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E43" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C44" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D44" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E44" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C45" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D45" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="E45" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C46" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D46" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E46" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C47" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D47" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E47" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C48" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D48" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E48" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C49" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D49" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="E49" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C50" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D50" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="E50" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C51" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D51" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E51" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C52" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D52" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="E52" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C53" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D53" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E53" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C54" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D54" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E54" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C55" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D55" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E55" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B56" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C56" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D56" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="E56" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B57" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C57" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D57" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E57" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C58" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D58" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="E58" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C59" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D59" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E59" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B60" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C60" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D60" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E60" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B61" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C61" t="n" s="2">
+        <v>45910.0</v>
+      </c>
+      <c r="D61" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E61" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B62" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C62" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D62" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E62" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B63" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C63" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D63" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="E63" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B64" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C64" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D64" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E64" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B65" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C65" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D65" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="E65" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B66" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C66" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D66" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E66" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B67" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C67" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D67" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E67" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B68" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C68" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D68" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E68" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B69" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C69" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D69" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E69" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B70" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C70" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D70" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E70" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B71" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C71" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D71" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E71" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B72" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C72" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D72" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E72" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B73" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C73" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D73" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E73" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B74" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C74" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D74" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E74" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B75" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C75" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D75" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="E75" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B76" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C76" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D76" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E76" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B77" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C77" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D77" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E77" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B78" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C78" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D78" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E78" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B79" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C79" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D79" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="E79" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B80" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C80" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D80" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="E80" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B81" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C81" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D81" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E81" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B82" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C82" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D82" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="E82" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B83" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C83" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D83" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E83" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B84" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C84" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D84" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E84" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B85" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C85" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D85" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E85" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B86" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C86" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D86" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="E86" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B87" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C87" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D87" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E87" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B88" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C88" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D88" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="E88" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B89" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C89" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D89" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E89" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B90" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C90" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D90" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E90" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B91" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C91" t="n" s="2">
+        <v>45917.0</v>
+      </c>
+      <c r="D91" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E91" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B92" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C92" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D92" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E92" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B93" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C93" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D93" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="E93" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B94" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C94" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D94" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E94" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B95" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C95" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D95" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="E95" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B96" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C96" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D96" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E96" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B97" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C97" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D97" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E97" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B98" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C98" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D98" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E98" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B99" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C99" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D99" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E99" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B100" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C100" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D100" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E100" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B101" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C101" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D101" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E101" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B102" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C102" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D102" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E102" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B103" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C103" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D103" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E103" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B104" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C104" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D104" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E104" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B105" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C105" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D105" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="E105" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B106" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C106" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D106" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E106" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B107" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C107" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D107" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E107" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B108" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C108" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D108" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E108" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B109" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C109" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D109" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="E109" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B110" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C110" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D110" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="E110" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B111" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C111" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D111" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E111" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B112" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C112" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D112" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="E112" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B113" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C113" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D113" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E113" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B114" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C114" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D114" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E114" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B115" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C115" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D115" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E115" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B116" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C116" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D116" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="E116" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B117" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C117" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D117" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E117" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B118" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C118" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D118" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="E118" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B119" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C119" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D119" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E119" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B120" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C120" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D120" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E120" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B121" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C121" t="n" s="2">
+        <v>45924.0</v>
+      </c>
+      <c r="D121" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E121" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Fixed Red Mark on startup program
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="49">
   <si>
     <t>ID</t>
   </si>
@@ -152,6 +152,15 @@
   </si>
   <si>
     <t>Присутствовал</t>
+  </si>
+  <si>
+    <t>Опоздал</t>
+  </si>
+  <si>
+    <t>Нет</t>
+  </si>
+  <si>
+    <t>Да</t>
   </si>
 </sst>
 </file>
@@ -390,7 +399,7 @@
         <v>4</v>
       </c>
       <c r="E6" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="7">
@@ -407,7 +416,7 @@
         <v>4</v>
       </c>
       <c r="E7" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="8">
@@ -424,7 +433,7 @@
         <v>4</v>
       </c>
       <c r="E8" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="9">
@@ -441,7 +450,7 @@
         <v>4</v>
       </c>
       <c r="E9" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="10">
@@ -893,13 +902,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="10.21875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="17.20703125" customWidth="true" bestFit="true"/>
-    <col min="3" max="3" width="5.44140625" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="14.10546875" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="9.92578125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="32.01953125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="14.71875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -920,6 +929,516 @@
         <v>45</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C2" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D2" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C3" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D3" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E3" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C4" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D4" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E4" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C5" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D5" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E5" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C6" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C7" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C8" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D8" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="E8" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C9" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D9" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E9" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C10" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D10" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E10" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C11" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C12" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C13" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C14" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C15" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D15" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E15" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C16" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D16" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E16" t="s" s="0">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C17" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D17" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E17" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C18" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D18" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E18" t="s" s="0">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C19" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D19" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E19" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C20" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D20" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E20" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C21" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D21" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="E21" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C22" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D22" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E22" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C23" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D23" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E23" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C24" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D24" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="E24" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C25" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D25" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E25" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B26" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C26" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D26" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="E26" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B27" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C27" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D27" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E27" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B28" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C28" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D28" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E28" t="s" s="0">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B29" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C29" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D29" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E29" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B30" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C30" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D30" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E30" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B31" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C31" t="n" s="2">
+        <v>45979.0</v>
+      </c>
+      <c r="D31" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E31" t="s" s="0">
+        <v>47</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Added comments and more other futures by Roman
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="263" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="495" uniqueCount="75">
   <si>
     <t>ID</t>
   </si>
@@ -25,12 +25,12 @@
     <t>Количество студентов</t>
   </si>
   <si>
+    <t>10702423</t>
+  </si>
+  <si>
     <t>10702323</t>
   </si>
   <si>
-    <t>10702423</t>
-  </si>
-  <si>
     <t>ID студента</t>
   </si>
   <si>
@@ -43,18 +43,6 @@
     <t>Посещений</t>
   </si>
   <si>
-    <t>Вика (Староста)</t>
-  </si>
-  <si>
-    <t>Кадебская Карина</t>
-  </si>
-  <si>
-    <t>Пивоварчик Максим</t>
-  </si>
-  <si>
-    <t>Пустошило Алексей</t>
-  </si>
-  <si>
     <t>Антоненко Дмитрий Евгеньевич</t>
   </si>
   <si>
@@ -143,6 +131,96 @@
   </si>
   <si>
     <t>Якубович Илья Михайлович</t>
+  </si>
+  <si>
+    <t>Амельянчик Александра Александровна</t>
+  </si>
+  <si>
+    <t>Астукевич Даниил Алексеевич</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Барановский Егор Игоревич  </t>
+  </si>
+  <si>
+    <t>Белуш Захар Сергеевич</t>
+  </si>
+  <si>
+    <t>Васько Андрей Александрович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Веремьёв Никита Владимирович  </t>
+  </si>
+  <si>
+    <t>Винник Алина Сергеевна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Винникова Виктория Максимовна </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Воробей Дмитрий Сергеевич  </t>
+  </si>
+  <si>
+    <t>Гузаревич Владислав Максимович</t>
+  </si>
+  <si>
+    <t>Демчук Никита Андреевич</t>
+  </si>
+  <si>
+    <t>Зинкевич Яна Витальевна</t>
+  </si>
+  <si>
+    <t>Иванов Роман Сергеевич</t>
+  </si>
+  <si>
+    <t>Кадебская Карина Сергеевна</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кардычкин Алексей Вадимович  </t>
+  </si>
+  <si>
+    <t>Качановский Назар Николаевич</t>
+  </si>
+  <si>
+    <t>Курьянчик Матвей Александрович</t>
+  </si>
+  <si>
+    <t>Кучинский Максим Алексеевич</t>
+  </si>
+  <si>
+    <t>Марковский Артем Генрихович</t>
+  </si>
+  <si>
+    <t>Найдун Александра Андреевна</t>
+  </si>
+  <si>
+    <t>Нехай Денис Сергеевич</t>
+  </si>
+  <si>
+    <t>Ничипор Ефим Михайлович</t>
+  </si>
+  <si>
+    <t>Пашик Святослав Владимирович</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Пивоварчик Максим Дмитриевич </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Политыко Андрей Владимирович  </t>
+  </si>
+  <si>
+    <t>Пупкевич Никита Вадимович</t>
+  </si>
+  <si>
+    <t>Пустошило Алексей Владимирович</t>
+  </si>
+  <si>
+    <t>Северина Анастасия Николаевна</t>
+  </si>
+  <si>
+    <t>Султанов Арсений Александрович</t>
+  </si>
+  <si>
+    <t>Третьяк Тимофей Николаевич</t>
   </si>
   <si>
     <t>Дата</t>
@@ -269,7 +347,7 @@
         <v>3</v>
       </c>
       <c r="C2" t="n" s="0">
-        <v>4.0</v>
+        <v>30.0</v>
       </c>
     </row>
     <row r="3">
@@ -290,11 +368,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="11.6171875" customWidth="true" bestFit="true"/>
-    <col min="2" max="2" width="32.01953125" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="35.07421875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.21875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="17.20703125" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="11.87890625" customWidth="true" bestFit="true"/>
@@ -348,7 +426,7 @@
         <v>3</v>
       </c>
       <c r="E3" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="4">
@@ -365,7 +443,7 @@
         <v>3</v>
       </c>
       <c r="E4" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="5">
@@ -382,7 +460,7 @@
         <v>3</v>
       </c>
       <c r="E5" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="6">
@@ -393,13 +471,13 @@
         <v>13</v>
       </c>
       <c r="C6" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E6" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="7">
@@ -410,13 +488,13 @@
         <v>14</v>
       </c>
       <c r="C7" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="8">
@@ -427,13 +505,13 @@
         <v>15</v>
       </c>
       <c r="C8" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E8" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="9">
@@ -444,13 +522,13 @@
         <v>16</v>
       </c>
       <c r="C9" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E9" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="10">
@@ -461,13 +539,13 @@
         <v>17</v>
       </c>
       <c r="C10" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="11">
@@ -478,13 +556,13 @@
         <v>18</v>
       </c>
       <c r="C11" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E11" t="n" s="0">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="12">
@@ -495,13 +573,13 @@
         <v>19</v>
       </c>
       <c r="C12" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E12" t="n" s="0">
-        <v>1.0</v>
+        <v>3.0</v>
       </c>
     </row>
     <row r="13">
@@ -512,13 +590,13 @@
         <v>20</v>
       </c>
       <c r="C13" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="14">
@@ -529,13 +607,13 @@
         <v>21</v>
       </c>
       <c r="C14" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E14" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="15">
@@ -546,10 +624,10 @@
         <v>22</v>
       </c>
       <c r="C15" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E15" t="n" s="0">
         <v>2.0</v>
@@ -563,13 +641,13 @@
         <v>23</v>
       </c>
       <c r="C16" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E16" t="n" s="0">
-        <v>2.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="17">
@@ -580,13 +658,13 @@
         <v>24</v>
       </c>
       <c r="C17" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="18">
@@ -597,13 +675,13 @@
         <v>25</v>
       </c>
       <c r="C18" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E18" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="19">
@@ -614,13 +692,13 @@
         <v>26</v>
       </c>
       <c r="C19" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E19" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="20">
@@ -631,13 +709,13 @@
         <v>27</v>
       </c>
       <c r="C20" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E20" t="n" s="0">
-        <v>0.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="21">
@@ -648,13 +726,13 @@
         <v>28</v>
       </c>
       <c r="C21" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="22">
@@ -665,13 +743,13 @@
         <v>29</v>
       </c>
       <c r="C22" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E22" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="23">
@@ -682,13 +760,13 @@
         <v>30</v>
       </c>
       <c r="C23" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E23" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="24">
@@ -699,13 +777,13 @@
         <v>31</v>
       </c>
       <c r="C24" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E24" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="25">
@@ -716,13 +794,13 @@
         <v>32</v>
       </c>
       <c r="C25" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="26">
@@ -733,13 +811,13 @@
         <v>33</v>
       </c>
       <c r="C26" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E26" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="27">
@@ -750,13 +828,13 @@
         <v>34</v>
       </c>
       <c r="C27" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E27" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="28">
@@ -767,13 +845,13 @@
         <v>35</v>
       </c>
       <c r="C28" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E28" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="29">
@@ -784,13 +862,13 @@
         <v>36</v>
       </c>
       <c r="C29" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E29" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="30">
@@ -801,10 +879,10 @@
         <v>37</v>
       </c>
       <c r="C30" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E30" t="n" s="0">
         <v>1.0</v>
@@ -818,13 +896,13 @@
         <v>38</v>
       </c>
       <c r="C31" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E31" t="n" s="0">
-        <v>1.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="32">
@@ -858,7 +936,7 @@
         <v>4</v>
       </c>
       <c r="E33" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
     </row>
     <row r="34">
@@ -875,7 +953,7 @@
         <v>4</v>
       </c>
       <c r="E34" t="n" s="0">
-        <v>0.0</v>
+        <v>1.0</v>
       </c>
     </row>
     <row r="35">
@@ -892,6 +970,448 @@
         <v>4</v>
       </c>
       <c r="E35" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n" s="0">
+        <v>34.0</v>
+      </c>
+      <c r="B36" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="C36" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D36" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E36" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n" s="0">
+        <v>35.0</v>
+      </c>
+      <c r="B37" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="C37" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D37" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E37" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n" s="0">
+        <v>36.0</v>
+      </c>
+      <c r="B38" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C38" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D38" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E38" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n" s="0">
+        <v>37.0</v>
+      </c>
+      <c r="B39" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="C39" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D39" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E39" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n" s="0">
+        <v>38.0</v>
+      </c>
+      <c r="B40" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="C40" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D40" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E40" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n" s="0">
+        <v>39.0</v>
+      </c>
+      <c r="B41" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="C41" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D41" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E41" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n" s="0">
+        <v>40.0</v>
+      </c>
+      <c r="B42" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="C42" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D42" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E42" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n" s="0">
+        <v>41.0</v>
+      </c>
+      <c r="B43" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="C43" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D43" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E43" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n" s="0">
+        <v>42.0</v>
+      </c>
+      <c r="B44" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="C44" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D44" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E44" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n" s="0">
+        <v>43.0</v>
+      </c>
+      <c r="B45" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="C45" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D45" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E45" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n" s="0">
+        <v>44.0</v>
+      </c>
+      <c r="B46" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="C46" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D46" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E46" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n" s="0">
+        <v>45.0</v>
+      </c>
+      <c r="B47" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="C47" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D47" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E47" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n" s="0">
+        <v>46.0</v>
+      </c>
+      <c r="B48" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="C48" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D48" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E48" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n" s="0">
+        <v>47.0</v>
+      </c>
+      <c r="B49" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="C49" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D49" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E49" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n" s="0">
+        <v>48.0</v>
+      </c>
+      <c r="B50" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="C50" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D50" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E50" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n" s="0">
+        <v>49.0</v>
+      </c>
+      <c r="B51" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="C51" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D51" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E51" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n" s="0">
+        <v>50.0</v>
+      </c>
+      <c r="B52" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="C52" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D52" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E52" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n" s="0">
+        <v>51.0</v>
+      </c>
+      <c r="B53" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="C53" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D53" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E53" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n" s="0">
+        <v>52.0</v>
+      </c>
+      <c r="B54" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="C54" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D54" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E54" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n" s="0">
+        <v>53.0</v>
+      </c>
+      <c r="B55" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="C55" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D55" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E55" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n" s="0">
+        <v>54.0</v>
+      </c>
+      <c r="B56" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="C56" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D56" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E56" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n" s="0">
+        <v>55.0</v>
+      </c>
+      <c r="B57" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="C57" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D57" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E57" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n" s="0">
+        <v>56.0</v>
+      </c>
+      <c r="B58" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="C58" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D58" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E58" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n" s="0">
+        <v>57.0</v>
+      </c>
+      <c r="B59" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="C59" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D59" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E59" t="n" s="0">
+        <v>1.0</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n" s="0">
+        <v>58.0</v>
+      </c>
+      <c r="B60" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="C60" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D60" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E60" t="n" s="0">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n" s="0">
+        <v>59.0</v>
+      </c>
+      <c r="B61" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="C61" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="D61" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="E61" t="n" s="0">
         <v>1.0</v>
       </c>
     </row>
@@ -902,13 +1422,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E61"/>
+  <dimension ref="A1:E121"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="10.21875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="17.20703125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="9.92578125" customWidth="true" bestFit="true"/>
-    <col min="4" max="4" width="32.01953125" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="35.07421875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="14.71875" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
@@ -920,310 +1440,310 @@
         <v>1</v>
       </c>
       <c r="C1" t="s" s="1">
-        <v>43</v>
+        <v>69</v>
       </c>
       <c r="D1" t="s" s="1">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="E1" t="s" s="1">
-        <v>45</v>
+        <v>71</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C7" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B8" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C8" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C9" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>46</v>
+        <v>73</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B10" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C10" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="E10" t="s" s="0">
-        <v>46</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C11" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>46</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C12" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C13" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>47</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B14" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C14" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="E14" t="s" s="0">
-        <v>47</v>
+        <v>72</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B15" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C15" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E15" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B16" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C16" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E16" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B17" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C17" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E17" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B18" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="E18" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B19" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C19" t="n" s="2">
         <v>45980.0</v>
@@ -1232,508 +1752,508 @@
         <v>31</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>47</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B20" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C20" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B21" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C21" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B22" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C22" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E22" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B23" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C23" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="E23" t="s" s="0">
-        <v>48</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B24" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C24" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>46</v>
+        <v>73</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B25" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C25" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="E25" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B26" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C26" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>48</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B27" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C27" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D27" t="s" s="0">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="E27" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B28" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C28" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="E28" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B29" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C29" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E29" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B30" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C30" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E30" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B31" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C31" t="n" s="2">
         <v>45980.0</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>28</v>
+        <v>14</v>
       </c>
       <c r="E31" t="s" s="0">
-        <v>46</v>
+        <v>72</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B32" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C32" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="E32" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B33" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C33" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="E33" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B34" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C34" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E34" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B35" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C35" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="E35" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B36" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C36" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>39</v>
+        <v>19</v>
       </c>
       <c r="E36" t="s" s="0">
-        <v>48</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B37" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C37" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>34</v>
+        <v>12</v>
       </c>
       <c r="E37" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B38" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C38" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>36</v>
+        <v>18</v>
       </c>
       <c r="E38" t="s" s="0">
-        <v>48</v>
+        <v>73</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B39" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C39" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E39" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B40" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C40" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B41" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C41" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B42" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C42" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="E42" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B43" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C43" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E43" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B44" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C44" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="E44" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B45" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C45" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E45" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B46" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C46" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="E46" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B47" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C47" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B48" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C48" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>46</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B49" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C49" t="n" s="2">
         <v>45987.0</v>
@@ -1742,211 +2262,1231 @@
         <v>31</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B50" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C50" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B51" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C51" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B52" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C52" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B53" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C53" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B54" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C54" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B55" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C55" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B56" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C56" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B57" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C57" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D57" t="s" s="0">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B58" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C58" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="E58" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B59" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C59" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>42</v>
+        <v>32</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>48</v>
+        <v>74</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B60" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C60" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>47</v>
+        <v>74</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="n" s="0">
-        <v>1.0</v>
+        <v>0.0</v>
       </c>
       <c r="B61" t="s" s="0">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C61" t="n" s="2">
         <v>45987.0</v>
       </c>
       <c r="D61" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E61" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B62" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C62" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D62" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="E62" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B63" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C63" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D63" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E63" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B64" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C64" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D64" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="E64" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B65" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C65" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D65" t="s" s="0">
         <v>28</v>
       </c>
-      <c r="E61" t="s" s="0">
+      <c r="E65" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B66" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C66" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D66" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="E66" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B67" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C67" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D67" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="E67" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B68" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C68" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D68" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="E68" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B69" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C69" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D69" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="E69" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B70" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C70" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D70" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="E70" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B71" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C71" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D71" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="E71" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B72" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C72" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D72" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="E72" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B73" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C73" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D73" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="E73" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B74" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C74" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D74" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E74" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B75" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C75" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D75" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="E75" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B76" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C76" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D76" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E76" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B77" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C77" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D77" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E77" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B78" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C78" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D78" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="E78" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B79" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C79" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D79" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E79" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B80" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C80" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D80" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="E80" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B81" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C81" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D81" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="E81" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B82" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C82" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D82" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="E82" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B83" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C83" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D83" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="E83" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B84" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C84" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D84" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="E84" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B85" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C85" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D85" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="E85" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B86" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C86" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D86" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="E86" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B87" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C87" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D87" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="E87" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B88" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C88" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D88" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="E88" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B89" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C89" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D89" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="E89" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B90" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C90" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D90" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="E90" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n" s="0">
+        <v>0.0</v>
+      </c>
+      <c r="B91" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="C91" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D91" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="E91" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B92" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C92" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D92" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="E92" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B93" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C93" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D93" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="E93" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B94" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C94" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D94" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="E94" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B95" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C95" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D95" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="E95" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B96" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C96" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D96" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="E96" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B97" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C97" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D97" t="s" s="0">
         <v>48</v>
+      </c>
+      <c r="E97" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B98" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C98" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D98" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="E98" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B99" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C99" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D99" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="E99" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B100" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C100" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D100" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="E100" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B101" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C101" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D101" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="E101" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B102" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C102" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D102" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="E102" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B103" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C103" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D103" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="E103" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B104" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C104" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D104" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="E104" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B105" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C105" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D105" t="s" s="0">
+        <v>53</v>
+      </c>
+      <c r="E105" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B106" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C106" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D106" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="E106" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B107" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C107" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D107" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="E107" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B108" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C108" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D108" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="E108" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B109" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C109" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D109" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="E109" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B110" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C110" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D110" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="E110" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B111" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C111" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D111" t="s" s="0">
+        <v>51</v>
+      </c>
+      <c r="E111" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B112" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C112" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D112" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="E112" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B113" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C113" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D113" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="E113" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B114" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C114" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D114" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="E114" t="s" s="0">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B115" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C115" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D115" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="E115" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B116" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C116" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D116" t="s" s="0">
+        <v>57</v>
+      </c>
+      <c r="E116" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B117" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C117" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D117" t="s" s="0">
+        <v>55</v>
+      </c>
+      <c r="E117" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B118" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C118" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D118" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="E118" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B119" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C119" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D119" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="E119" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B120" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C120" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D120" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E120" t="s" s="0">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n" s="0">
+        <v>1.0</v>
+      </c>
+      <c r="B121" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C121" t="n" s="2">
+        <v>45992.0</v>
+      </c>
+      <c r="D121" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="E121" t="s" s="0">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Version 1.9 by @Roman
</commit_message>
<xml_diff>
--- a/attendance_data.xlsx
+++ b/attendance_data.xlsx
@@ -235,10 +235,10 @@
     <t>Да</t>
   </si>
   <si>
+    <t>Нет</t>
+  </si>
+  <si>
     <t>Опоздал</t>
-  </si>
-  <si>
-    <t>Нет</t>
   </si>
 </sst>
 </file>
@@ -1460,7 +1460,7 @@
         <v>45980.0</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E2" t="s" s="0">
         <v>72</v>
@@ -1477,10 +1477,10 @@
         <v>45980.0</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4">
@@ -1494,7 +1494,7 @@
         <v>45980.0</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E4" t="s" s="0">
         <v>72</v>
@@ -1511,7 +1511,7 @@
         <v>45980.0</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E5" t="s" s="0">
         <v>72</v>
@@ -1528,7 +1528,7 @@
         <v>45980.0</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E6" t="s" s="0">
         <v>72</v>
@@ -1545,7 +1545,7 @@
         <v>45980.0</v>
       </c>
       <c r="D7" t="s" s="0">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="E7" t="s" s="0">
         <v>72</v>
@@ -1562,10 +1562,10 @@
         <v>45980.0</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E8" t="s" s="0">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9">
@@ -1579,7 +1579,7 @@
         <v>45980.0</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E9" t="s" s="0">
         <v>73</v>
@@ -1596,7 +1596,7 @@
         <v>45980.0</v>
       </c>
       <c r="D10" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E10" t="s" s="0">
         <v>74</v>
@@ -1613,10 +1613,10 @@
         <v>45980.0</v>
       </c>
       <c r="D11" t="s" s="0">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="12">
@@ -1630,7 +1630,7 @@
         <v>45980.0</v>
       </c>
       <c r="D12" t="s" s="0">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E12" t="s" s="0">
         <v>72</v>
@@ -1647,7 +1647,7 @@
         <v>45980.0</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E13" t="s" s="0">
         <v>72</v>
@@ -1664,7 +1664,7 @@
         <v>45980.0</v>
       </c>
       <c r="D14" t="s" s="0">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="E14" t="s" s="0">
         <v>72</v>
@@ -1681,7 +1681,7 @@
         <v>45980.0</v>
       </c>
       <c r="D15" t="s" s="0">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E15" t="s" s="0">
         <v>72</v>
@@ -1698,7 +1698,7 @@
         <v>45980.0</v>
       </c>
       <c r="D16" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E16" t="s" s="0">
         <v>72</v>
@@ -1715,7 +1715,7 @@
         <v>45980.0</v>
       </c>
       <c r="D17" t="s" s="0">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E17" t="s" s="0">
         <v>72</v>
@@ -1732,7 +1732,7 @@
         <v>45980.0</v>
       </c>
       <c r="D18" t="s" s="0">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E18" t="s" s="0">
         <v>72</v>
@@ -1749,10 +1749,10 @@
         <v>45980.0</v>
       </c>
       <c r="D19" t="s" s="0">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E19" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20">
@@ -1766,10 +1766,10 @@
         <v>45980.0</v>
       </c>
       <c r="D20" t="s" s="0">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="E20" t="s" s="0">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21">
@@ -1783,10 +1783,10 @@
         <v>45980.0</v>
       </c>
       <c r="D21" t="s" s="0">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E21" t="s" s="0">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="22">
@@ -1800,7 +1800,7 @@
         <v>45980.0</v>
       </c>
       <c r="D22" t="s" s="0">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E22" t="s" s="0">
         <v>72</v>
@@ -1817,7 +1817,7 @@
         <v>45980.0</v>
       </c>
       <c r="D23" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E23" t="s" s="0">
         <v>72</v>
@@ -1834,10 +1834,10 @@
         <v>45980.0</v>
       </c>
       <c r="D24" t="s" s="0">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E24" t="s" s="0">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="25">
@@ -1851,7 +1851,7 @@
         <v>45980.0</v>
       </c>
       <c r="D25" t="s" s="0">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E25" t="s" s="0">
         <v>72</v>
@@ -1868,10 +1868,10 @@
         <v>45980.0</v>
       </c>
       <c r="D26" t="s" s="0">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E26" t="s" s="0">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="27">
@@ -1902,7 +1902,7 @@
         <v>45980.0</v>
       </c>
       <c r="D28" t="s" s="0">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E28" t="s" s="0">
         <v>72</v>
@@ -1919,10 +1919,10 @@
         <v>45980.0</v>
       </c>
       <c r="D29" t="s" s="0">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="E29" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="30">
@@ -1936,7 +1936,7 @@
         <v>45980.0</v>
       </c>
       <c r="D30" t="s" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E30" t="s" s="0">
         <v>72</v>
@@ -1953,7 +1953,7 @@
         <v>45980.0</v>
       </c>
       <c r="D31" t="s" s="0">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E31" t="s" s="0">
         <v>72</v>
@@ -1970,10 +1970,10 @@
         <v>45987.0</v>
       </c>
       <c r="D32" t="s" s="0">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E32" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="33">
@@ -1987,10 +1987,10 @@
         <v>45987.0</v>
       </c>
       <c r="D33" t="s" s="0">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="E33" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="34">
@@ -2004,10 +2004,10 @@
         <v>45987.0</v>
       </c>
       <c r="D34" t="s" s="0">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E34" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="35">
@@ -2021,7 +2021,7 @@
         <v>45987.0</v>
       </c>
       <c r="D35" t="s" s="0">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E35" t="s" s="0">
         <v>74</v>
@@ -2038,10 +2038,10 @@
         <v>45987.0</v>
       </c>
       <c r="D36" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E36" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="37">
@@ -2055,10 +2055,10 @@
         <v>45987.0</v>
       </c>
       <c r="D37" t="s" s="0">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="E37" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="38">
@@ -2072,7 +2072,7 @@
         <v>45987.0</v>
       </c>
       <c r="D38" t="s" s="0">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E38" t="s" s="0">
         <v>73</v>
@@ -2089,10 +2089,10 @@
         <v>45987.0</v>
       </c>
       <c r="D39" t="s" s="0">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E39" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40">
@@ -2106,10 +2106,10 @@
         <v>45987.0</v>
       </c>
       <c r="D40" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E40" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="41">
@@ -2123,10 +2123,10 @@
         <v>45987.0</v>
       </c>
       <c r="D41" t="s" s="0">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="E41" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="42">
@@ -2140,10 +2140,10 @@
         <v>45987.0</v>
       </c>
       <c r="D42" t="s" s="0">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E42" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="43">
@@ -2157,10 +2157,10 @@
         <v>45987.0</v>
       </c>
       <c r="D43" t="s" s="0">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E43" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="44">
@@ -2174,10 +2174,10 @@
         <v>45987.0</v>
       </c>
       <c r="D44" t="s" s="0">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="E44" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="45">
@@ -2191,10 +2191,10 @@
         <v>45987.0</v>
       </c>
       <c r="D45" t="s" s="0">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E45" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="46">
@@ -2208,10 +2208,10 @@
         <v>45987.0</v>
       </c>
       <c r="D46" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E46" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="47">
@@ -2225,10 +2225,10 @@
         <v>45987.0</v>
       </c>
       <c r="D47" t="s" s="0">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E47" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="48">
@@ -2242,10 +2242,10 @@
         <v>45987.0</v>
       </c>
       <c r="D48" t="s" s="0">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E48" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49">
@@ -2259,10 +2259,10 @@
         <v>45987.0</v>
       </c>
       <c r="D49" t="s" s="0">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E49" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="50">
@@ -2276,10 +2276,10 @@
         <v>45987.0</v>
       </c>
       <c r="D50" t="s" s="0">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="E50" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="51">
@@ -2293,10 +2293,10 @@
         <v>45987.0</v>
       </c>
       <c r="D51" t="s" s="0">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E51" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="52">
@@ -2310,10 +2310,10 @@
         <v>45987.0</v>
       </c>
       <c r="D52" t="s" s="0">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E52" t="s" s="0">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="53">
@@ -2327,10 +2327,10 @@
         <v>45987.0</v>
       </c>
       <c r="D53" t="s" s="0">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E53" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="54">
@@ -2344,10 +2344,10 @@
         <v>45987.0</v>
       </c>
       <c r="D54" t="s" s="0">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E54" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="55">
@@ -2361,10 +2361,10 @@
         <v>45987.0</v>
       </c>
       <c r="D55" t="s" s="0">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E55" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="56">
@@ -2378,10 +2378,10 @@
         <v>45987.0</v>
       </c>
       <c r="D56" t="s" s="0">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E56" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="57">
@@ -2398,7 +2398,7 @@
         <v>13</v>
       </c>
       <c r="E57" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="58">
@@ -2412,10 +2412,10 @@
         <v>45987.0</v>
       </c>
       <c r="D58" t="s" s="0">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E58" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="59">
@@ -2429,10 +2429,10 @@
         <v>45987.0</v>
       </c>
       <c r="D59" t="s" s="0">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="E59" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="60">
@@ -2446,10 +2446,10 @@
         <v>45987.0</v>
       </c>
       <c r="D60" t="s" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E60" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="61">
@@ -2463,10 +2463,10 @@
         <v>45987.0</v>
       </c>
       <c r="D61" t="s" s="0">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E61" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="62">
@@ -2480,7 +2480,7 @@
         <v>45992.0</v>
       </c>
       <c r="D62" t="s" s="0">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E62" t="s" s="0">
         <v>72</v>
@@ -2497,7 +2497,7 @@
         <v>45992.0</v>
       </c>
       <c r="D63" t="s" s="0">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="E63" t="s" s="0">
         <v>72</v>
@@ -2514,7 +2514,7 @@
         <v>45992.0</v>
       </c>
       <c r="D64" t="s" s="0">
-        <v>36</v>
+        <v>12</v>
       </c>
       <c r="E64" t="s" s="0">
         <v>72</v>
@@ -2531,10 +2531,10 @@
         <v>45992.0</v>
       </c>
       <c r="D65" t="s" s="0">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="E65" t="s" s="0">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="66">
@@ -2548,7 +2548,7 @@
         <v>45992.0</v>
       </c>
       <c r="D66" t="s" s="0">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E66" t="s" s="0">
         <v>72</v>
@@ -2565,7 +2565,7 @@
         <v>45992.0</v>
       </c>
       <c r="D67" t="s" s="0">
-        <v>12</v>
+        <v>38</v>
       </c>
       <c r="E67" t="s" s="0">
         <v>72</v>
@@ -2582,7 +2582,7 @@
         <v>45992.0</v>
       </c>
       <c r="D68" t="s" s="0">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="E68" t="s" s="0">
         <v>72</v>
@@ -2599,10 +2599,10 @@
         <v>45992.0</v>
       </c>
       <c r="D69" t="s" s="0">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="E69" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="70">
@@ -2616,7 +2616,7 @@
         <v>45992.0</v>
       </c>
       <c r="D70" t="s" s="0">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E70" t="s" s="0">
         <v>74</v>
@@ -2633,7 +2633,7 @@
         <v>45992.0</v>
       </c>
       <c r="D71" t="s" s="0">
-        <v>9</v>
+        <v>28</v>
       </c>
       <c r="E71" t="s" s="0">
         <v>74</v>
@@ -2650,10 +2650,10 @@
         <v>45992.0</v>
       </c>
       <c r="D72" t="s" s="0">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E72" t="s" s="0">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="73">
@@ -2667,7 +2667,7 @@
         <v>45992.0</v>
       </c>
       <c r="D73" t="s" s="0">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="E73" t="s" s="0">
         <v>72</v>
@@ -2684,7 +2684,7 @@
         <v>45992.0</v>
       </c>
       <c r="D74" t="s" s="0">
-        <v>38</v>
+        <v>21</v>
       </c>
       <c r="E74" t="s" s="0">
         <v>72</v>
@@ -2701,10 +2701,10 @@
         <v>45992.0</v>
       </c>
       <c r="D75" t="s" s="0">
-        <v>25</v>
+        <v>33</v>
       </c>
       <c r="E75" t="s" s="0">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="76">
@@ -2718,7 +2718,7 @@
         <v>45992.0</v>
       </c>
       <c r="D76" t="s" s="0">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="E76" t="s" s="0">
         <v>72</v>
@@ -2735,7 +2735,7 @@
         <v>45992.0</v>
       </c>
       <c r="D77" t="s" s="0">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="E77" t="s" s="0">
         <v>72</v>
@@ -2752,10 +2752,10 @@
         <v>45992.0</v>
       </c>
       <c r="D78" t="s" s="0">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="E78" t="s" s="0">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="79">
@@ -2769,10 +2769,10 @@
         <v>45992.0</v>
       </c>
       <c r="D79" t="s" s="0">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="E79" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="80">
@@ -2786,7 +2786,7 @@
         <v>45992.0</v>
       </c>
       <c r="D80" t="s" s="0">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="E80" t="s" s="0">
         <v>72</v>
@@ -2803,7 +2803,7 @@
         <v>45992.0</v>
       </c>
       <c r="D81" t="s" s="0">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E81" t="s" s="0">
         <v>72</v>
@@ -2820,7 +2820,7 @@
         <v>45992.0</v>
       </c>
       <c r="D82" t="s" s="0">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="E82" t="s" s="0">
         <v>72</v>
@@ -2837,7 +2837,7 @@
         <v>45992.0</v>
       </c>
       <c r="D83" t="s" s="0">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="E83" t="s" s="0">
         <v>72</v>
@@ -2854,7 +2854,7 @@
         <v>45992.0</v>
       </c>
       <c r="D84" t="s" s="0">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="E84" t="s" s="0">
         <v>72</v>
@@ -2871,7 +2871,7 @@
         <v>45992.0</v>
       </c>
       <c r="D85" t="s" s="0">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E85" t="s" s="0">
         <v>72</v>
@@ -2888,10 +2888,10 @@
         <v>45992.0</v>
       </c>
       <c r="D86" t="s" s="0">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E86" t="s" s="0">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="87">
@@ -2922,7 +2922,7 @@
         <v>45992.0</v>
       </c>
       <c r="D88" t="s" s="0">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="E88" t="s" s="0">
         <v>72</v>
@@ -2939,10 +2939,10 @@
         <v>45992.0</v>
       </c>
       <c r="D89" t="s" s="0">
-        <v>32</v>
+        <v>11</v>
       </c>
       <c r="E89" t="s" s="0">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="90">
@@ -2956,7 +2956,7 @@
         <v>45992.0</v>
       </c>
       <c r="D90" t="s" s="0">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="E90" t="s" s="0">
         <v>72</v>
@@ -2973,7 +2973,7 @@
         <v>45992.0</v>
       </c>
       <c r="D91" t="s" s="0">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E91" t="s" s="0">
         <v>72</v>
@@ -2990,10 +2990,10 @@
         <v>45992.0</v>
       </c>
       <c r="D92" t="s" s="0">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E92" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="93">
@@ -3007,10 +3007,10 @@
         <v>45992.0</v>
       </c>
       <c r="D93" t="s" s="0">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="E93" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="94">
@@ -3024,10 +3024,10 @@
         <v>45992.0</v>
       </c>
       <c r="D94" t="s" s="0">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E94" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="95">
@@ -3041,10 +3041,10 @@
         <v>45992.0</v>
       </c>
       <c r="D95" t="s" s="0">
-        <v>46</v>
+        <v>62</v>
       </c>
       <c r="E95" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="96">
@@ -3058,10 +3058,10 @@
         <v>45992.0</v>
       </c>
       <c r="D96" t="s" s="0">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="E96" t="s" s="0">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="97">
@@ -3075,10 +3075,10 @@
         <v>45992.0</v>
       </c>
       <c r="D97" t="s" s="0">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E97" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="98">
@@ -3092,10 +3092,10 @@
         <v>45992.0</v>
       </c>
       <c r="D98" t="s" s="0">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E98" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="99">
@@ -3109,10 +3109,10 @@
         <v>45992.0</v>
       </c>
       <c r="D99" t="s" s="0">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E99" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="100">
@@ -3126,7 +3126,7 @@
         <v>45992.0</v>
       </c>
       <c r="D100" t="s" s="0">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E100" t="s" s="0">
         <v>73</v>
@@ -3143,7 +3143,7 @@
         <v>45992.0</v>
       </c>
       <c r="D101" t="s" s="0">
-        <v>43</v>
+        <v>65</v>
       </c>
       <c r="E101" t="s" s="0">
         <v>72</v>
@@ -3160,10 +3160,10 @@
         <v>45992.0</v>
       </c>
       <c r="D102" t="s" s="0">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="E102" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="103">
@@ -3177,10 +3177,10 @@
         <v>45992.0</v>
       </c>
       <c r="D103" t="s" s="0">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="E103" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="104">
@@ -3194,10 +3194,10 @@
         <v>45992.0</v>
       </c>
       <c r="D104" t="s" s="0">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="E104" t="s" s="0">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="105">
@@ -3211,10 +3211,10 @@
         <v>45992.0</v>
       </c>
       <c r="D105" t="s" s="0">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E105" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="106">
@@ -3228,10 +3228,10 @@
         <v>45992.0</v>
       </c>
       <c r="D106" t="s" s="0">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E106" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="107">
@@ -3245,10 +3245,10 @@
         <v>45992.0</v>
       </c>
       <c r="D107" t="s" s="0">
-        <v>39</v>
+        <v>66</v>
       </c>
       <c r="E107" t="s" s="0">
-        <v>72</v>
+        <v>74</v>
       </c>
     </row>
     <row r="108">
@@ -3262,7 +3262,7 @@
         <v>45992.0</v>
       </c>
       <c r="D108" t="s" s="0">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="E108" t="s" s="0">
         <v>74</v>
@@ -3296,10 +3296,10 @@
         <v>45992.0</v>
       </c>
       <c r="D110" t="s" s="0">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="E110" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="111">
@@ -3313,10 +3313,10 @@
         <v>45992.0</v>
       </c>
       <c r="D111" t="s" s="0">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="E111" t="s" s="0">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="112">
@@ -3330,10 +3330,10 @@
         <v>45992.0</v>
       </c>
       <c r="D112" t="s" s="0">
-        <v>41</v>
+        <v>63</v>
       </c>
       <c r="E112" t="s" s="0">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="113">
@@ -3347,7 +3347,7 @@
         <v>45992.0</v>
       </c>
       <c r="D113" t="s" s="0">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="E113" t="s" s="0">
         <v>73</v>
@@ -3364,10 +3364,10 @@
         <v>45992.0</v>
       </c>
       <c r="D114" t="s" s="0">
-        <v>42</v>
+        <v>55</v>
       </c>
       <c r="E114" t="s" s="0">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="115">
@@ -3381,10 +3381,10 @@
         <v>45992.0</v>
       </c>
       <c r="D115" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="E115" t="s" s="0">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="116">
@@ -3398,10 +3398,10 @@
         <v>45992.0</v>
       </c>
       <c r="D116" t="s" s="0">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="E116" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="117">
@@ -3415,10 +3415,10 @@
         <v>45992.0</v>
       </c>
       <c r="D117" t="s" s="0">
-        <v>55</v>
+        <v>67</v>
       </c>
       <c r="E117" t="s" s="0">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="118">
@@ -3432,10 +3432,10 @@
         <v>45992.0</v>
       </c>
       <c r="D118" t="s" s="0">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="E118" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="119">
@@ -3449,7 +3449,7 @@
         <v>45992.0</v>
       </c>
       <c r="D119" t="s" s="0">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E119" t="s" s="0">
         <v>74</v>
@@ -3466,10 +3466,10 @@
         <v>45992.0</v>
       </c>
       <c r="D120" t="s" s="0">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="E120" t="s" s="0">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="121">
@@ -3483,10 +3483,10 @@
         <v>45992.0</v>
       </c>
       <c r="D121" t="s" s="0">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E121" t="s" s="0">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>